<commit_message>
docs: regenerate deliverables for v1.42.0 (all PM packages)
- Excel export: +10 register sheets (change requests, issues, stakeholders,
  decisions, impediments, lessons, RACI, story map, poker, portfolio) -> 40 sheets.
- Docx: 13 new sections in description/illustrated (with screenshots), a "18. PM
  practices" chapter in the user guide, V10 notes in admin/deploy guides; version 1.42.0.
- PPTX: +7 slides (EVM, stakeholders, WBS, story map, poker, portfolio, status report) -> 49.
- Chat assistant keywords for the new sections.
Frontend e2e 87/87, backend 7/7.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Планирование_спринта_PRO.xlsx
+++ b/Планирование_спринта_PRO.xlsx
@@ -32,6 +32,16 @@
     <sheet name="График отпусков" sheetId="28" r:id="rId28"/>
     <sheet name="Дни рождения" sheetId="29" r:id="rId29"/>
     <sheet name="Контроль scope" sheetId="30" r:id="rId30"/>
+    <sheet name="Запросы на изменение" sheetId="31" r:id="rId31"/>
+    <sheet name="Журнал проблем" sheetId="32" r:id="rId32"/>
+    <sheet name="Стейкхолдеры" sheetId="33" r:id="rId33"/>
+    <sheet name="Журнал решений" sheetId="34" r:id="rId34"/>
+    <sheet name="Импедименты" sheetId="35" r:id="rId35"/>
+    <sheet name="Уроки" sheetId="36" r:id="rId36"/>
+    <sheet name="RACI" sheetId="37" r:id="rId37"/>
+    <sheet name="Story Map" sheetId="38" r:id="rId38"/>
+    <sheet name="Planning Poker" sheetId="39" r:id="rId39"/>
+    <sheet name="Портфель" sheetId="40" r:id="rId40"/>
   </sheets>
 </workbook>
 </file>
@@ -6491,6 +6501,112 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E-1</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Эпик: Оформление и оплата заказа</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Эпик</t>
+        </is>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">В работе</t>
+        </is>
+      </c>
+      <c r="H22">
+        <v>0</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E-2</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Эпик: Каталог и личный кабинет</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Эпик</t>
+        </is>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">To Do</t>
+        </is>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -6594,6 +6710,1526 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Дата</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Запрос</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Тип</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Влияние</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Инициатор</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Статус</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Решение</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CR-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-30</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Добавить вход через SSO (OAuth2)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scope</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+8 SP, +1 спринт</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Product Owner</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Одобрен</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Включено в релиз R-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CR-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Поддержка оплаты в рассрочку</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scope</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+13 SP</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Коммерция</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Отложен</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Вернуться после MVP</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CR-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-14</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Сдвиг даты релиза на 2 недели</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Срок</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">−1 риск, −ценность</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Спонсор</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Предложен</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Нужно решение CCB</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Дата</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Проблема</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Приоритет</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Владелец</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Статус</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Срок</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Решение</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IS-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-05</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Платёжный шлюз возвращает таймауты в песочнице</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Кузнецов Д.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">В работе</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-20</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Эскалировано провайдеру</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IS-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Расхождение остатков каталога с 1С</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Орлова Е.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Открыта</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-25</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IS-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-28</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Падение сборки CI на флейки-тестах</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DevOps</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Решена</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-02</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Карантин флейки-тестов</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Стейкхолдер</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Роль</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Влияние</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Интерес</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Вовлечённость</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Целевая</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Стратегия</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SH-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Директор по продукту</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Спонсор</t>
+        </is>
+      </c>
+      <c r="D2">
+        <v>5</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Поддерживающий</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лидер</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Еженедельный статус + демо</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SH-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Финансовый директор</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Бюджет</t>
+        </is>
+      </c>
+      <c r="D3">
+        <v>5</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Нейтральный</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Поддерживающий</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Держать удовлетворённым: отчёт по бюджету</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SH-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Служба поддержки</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Операции</t>
+        </is>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4">
+        <v>4</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Поддерживающий</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Поддерживающий</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Информировать о релизах</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SH-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Отдел безопасности</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Compliance</t>
+        </is>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
+      <c r="E5">
+        <v>3</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Сопротивляется</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Нейтральный</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ранние ревью, PCI DSS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SH-05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Маркетинг</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Go-to-market</t>
+        </is>
+      </c>
+      <c r="D6">
+        <v>3</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Поддерживающий</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лидер</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Совместное планирование запуска</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Дата</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Решение</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Контекст</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Варианты</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Что решили</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Обоснование</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Владелец</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Статус</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DC-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-12</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PostgreSQL как основная СУБД</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Нужны транзакции и отчётность</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PostgreSQL / MongoDB</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PostgreSQL</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ACID, зрелость, SQL-аналитика</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Архитектор</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Принято</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DC-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-20</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Двухнедельные спринты</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Баланс обратной связи и накладных</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 / 2 / 3 недели</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 недели</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Оптимальный ритм для команды</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scrum-мастер</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Принято</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DC-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-10</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Платёжный провайдер</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Выбор интеграции оплаты</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Провайдер A / B</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Провайдер A (пилот)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Быстрее интеграция, тест-режим</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Product Owner</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Пересмотрено</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Возник</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Импедимент</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Владелец</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Серьёзность</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Статус</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Спринт</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Снят</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IM-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Нет ключей от платёжного провайдера</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Product Owner</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">В работе</t>
+        </is>
+      </c>
+      <c r="G2">
+        <v>3</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IM-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-12</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Стенд нестабилен (падает ночью)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DevOps</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Открыт</t>
+        </is>
+      </c>
+      <c r="G3">
+        <v>3</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Дата</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Спринт</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Категория</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ситуация</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Урок</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Рекомендация</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LE-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-29</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Процесс</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Недооценили интеграцию оплаты</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Для внешних интеграций нужен спайк</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Добавлять исследовательскую задачу и буфер</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LE-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-12</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>3</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Качество</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Флейки-тесты роняли CI</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Нестабильные тесты дороже, чем кажется</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Карантин флейки-тестов и починка по SLA</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Активность</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RA-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Планирование спринта</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Команда</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scrum-мастер</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Product Owner</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Стейкхолдеры</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RA-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Приоритизация бэклога</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Product Owner</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Product Owner</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Команда</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ИТ-Лидер</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RA-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Релиз в прод</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DevOps</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ИТ-Лидер</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Поддержка, PO</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RA-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Приёмка на демо</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Product Owner</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Product Owner</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Команда</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Заказчик</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Активность</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Релиз</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">История</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Задача</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SM-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Выбор товара</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R-1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Каталог и карточка товара</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SM-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Корзина</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R-1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Добавление и редактирование корзины</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SM-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Оформление</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R-1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Оформление заказа (MVP)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SM-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Оплата</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R-1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Оплата картой</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SM-05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Оформление</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R-2</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Промокоды и скидки</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SM-06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Оплата</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R-2</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Оплата в рассрочку</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SM-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">После покупки</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R-2</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">История заказов и уведомления</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Задача</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">История</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Голоса</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Итог</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Статус</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T-03</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Оплата картой</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Иванов:5, Петрова:8, Кузнецов:8, Орлова:5</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Завершён</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PK-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Промокоды и скидки</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Иванов:3, Петрова:5, Кузнецов:8</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Открыт</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetData>
@@ -6851,6 +8487,191 @@
       </c>
       <c r="D14">
         <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Проект</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RAG</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Health</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Velocity</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Бюджет</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Потрачено</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Прогресс</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Владелец</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Комментарий</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PO-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Маркетплейс (текущий)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Жёлтый</t>
+        </is>
+      </c>
+      <c r="D2">
+        <v>0.62</v>
+      </c>
+      <c r="E2">
+        <v>34</v>
+      </c>
+      <c r="F2">
+        <v>8000000</v>
+      </c>
+      <c r="G2">
+        <v>3200000</v>
+      </c>
+      <c r="H2">
+        <v>0.45</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PMO</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Активный проект</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PO-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Мобильное приложение</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Зелёный</t>
+        </is>
+      </c>
+      <c r="D3">
+        <v>0.82</v>
+      </c>
+      <c r="E3">
+        <v>28</v>
+      </c>
+      <c r="F3">
+        <v>5000000</v>
+      </c>
+      <c r="G3">
+        <v>1500000</v>
+      </c>
+      <c r="H3">
+        <v>0.3</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mobile Lead</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">По плану</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PO-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Миграция в облако</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Красный</t>
+        </is>
+      </c>
+      <c r="D4">
+        <v>0.48</v>
+      </c>
+      <c r="E4">
+        <v>18</v>
+      </c>
+      <c r="F4">
+        <v>6000000</v>
+      </c>
+      <c r="G4">
+        <v>4800000</v>
+      </c>
+      <c r="H4">
+        <v>0.7</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Platform</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Перерасход, риск сроков</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: regenerate deliverables for v1.43.0 (team health & performance)
- Docx: 4 new sections (Bus factor, Team Health Check, DORA, Incidents) in description/
  illustrated (+screenshots), «19. Health & performance» chapter in the user guide, V11
  notes in admin/deploy; version 1.43.0.
- PPTX: +4 slides (53 total, «Итог» kept last).
- Excel: +3 register sheets (team health, deployments, incidents) -> 43 sheets.
- Synced frontend/docs (Support downloads).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Планирование_спринта_PRO.xlsx
+++ b/Планирование_спринта_PRO.xlsx
@@ -42,6 +42,9 @@
     <sheet name="Story Map" sheetId="38" r:id="rId38"/>
     <sheet name="Planning Poker" sheetId="39" r:id="rId39"/>
     <sheet name="Портфель" sheetId="40" r:id="rId40"/>
+    <sheet name="Team Health Check" sheetId="41" r:id="rId41"/>
+    <sheet name="Деплои" sheetId="42" r:id="rId42"/>
+    <sheet name="Инциденты" sheetId="43" r:id="rId43"/>
   </sheets>
 </workbook>
 </file>
@@ -8678,6 +8681,858 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Дата</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Спринт</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Измерение</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Оценка</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Тренд</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Комментарий</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HC-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-11</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Поставка ценности</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Зелёный</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Растёт</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Регулярные демо принимаются</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HC-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-11</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>3</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Простота работы</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Жёлтый</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Стабильно</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Много ручной рутины</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HC-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-11</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Обучение</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Зелёный</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Растёт</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Парное программирование</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HC-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-11</t>
+        </is>
+      </c>
+      <c r="C5">
+        <v>3</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Миссия</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Зелёный</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Стабильно</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Цель понятна всем</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HC-05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-11</t>
+        </is>
+      </c>
+      <c r="C6">
+        <v>3</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Командная работа</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Зелёный</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Растёт</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Хорошая взаимопомощь</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HC-06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-11</t>
+        </is>
+      </c>
+      <c r="C7">
+        <v>3</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Поддержка и помощь</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Жёлтый</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Стабильно</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Внешние зависимости тормозят</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HC-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-11</t>
+        </is>
+      </c>
+      <c r="C8">
+        <v>3</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Пешки или игроки</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Зелёный</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Стабильно</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Команда влияет на решения</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HC-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-11</t>
+        </is>
+      </c>
+      <c r="C9">
+        <v>3</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Скорость</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Жёлтый</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Падает</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Блокеры по оплате</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HC-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-11</t>
+        </is>
+      </c>
+      <c r="C10">
+        <v>3</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Подходящий процесс</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Зелёный</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Стабильно</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scrum устоялся</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HC-10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-11</t>
+        </is>
+      </c>
+      <c r="C11">
+        <v>3</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Здоровье кодовой базы</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Красный</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Падает</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Рост техдолга и флейки-тестов</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HC-11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-11</t>
+        </is>
+      </c>
+      <c r="C12">
+        <v>3</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Весело</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Зелёный</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Стабильно</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Команда мотивирована</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Дата</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Релиз</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Среда</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Статус</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lead time (дн)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Комментарий</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DP-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-15</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R-1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prod</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Успех</t>
+        </is>
+      </c>
+      <c r="F2">
+        <v>3</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Каркас каталога</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DP-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-27</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R-1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prod</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Успех</t>
+        </is>
+      </c>
+      <c r="F3">
+        <v>2.2</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Корзина</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DP-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-02</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R-1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stage</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Успех</t>
+        </is>
+      </c>
+      <c r="F4">
+        <v>1.4</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Оплата (пилот)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DP-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R-1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prod</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Откат</t>
+        </is>
+      </c>
+      <c r="F5">
+        <v>2.8</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Откат из-за сбоя оплаты</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DP-05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-10</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R-1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prod</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Успех</t>
+        </is>
+      </c>
+      <c r="F6">
+        <v>0.6</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Хотфикс оплаты</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DP-06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-14</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R-2</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prod</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Успех</t>
+        </is>
+      </c>
+      <c r="F7">
+        <v>1.9</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Уведомления</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Дата</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Инцидент</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Серьёзность</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Восстановление (ч)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Причина</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Статус</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Постмортем</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IN-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Массовые таймауты оплаты в проде</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Critical</t>
+        </is>
+      </c>
+      <c r="E2">
+        <v>2.5</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Таймаут платёжного шлюза</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Восстановлен</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Добавить ретраи и circuit breaker</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IN-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-12</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Расхождение остатков каталога</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="E3">
+        <v>6</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Задержка синхронизации с 1С</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Закрыт</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Мониторинг лага синхронизации</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IN-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-15</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Падение уведомлений (email)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>1.2</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лимит SMTP</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Восстановлен</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Очередь и бэкофф</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetData>

</xml_diff>